<commit_message>
don't consider biometric in attendance, only maintaining count, and added shedulinh using airflow
</commit_message>
<xml_diff>
--- a/email_detials/employees_email_ID.xlsx
+++ b/email_detials/employees_email_ID.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\PRESENCE PRO 2.O\email_detials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985F3037-2132-4A71-A3B2-CBB4EBB94F73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5552E9E5-38CB-4B3C-9E95-CEA941D8ACBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Employees Master Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>NucleusTeq</t>
   </si>
@@ -616,7 +616,9 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="B7" s="5"/>
+      <c r="B7" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
removed biometric files and features, now we are sending email and consolidated file using Employee Number as index
</commit_message>
<xml_diff>
--- a/email_detials/employees_email_ID.xlsx
+++ b/email_detials/employees_email_ID.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\PRESENCE PRO 2.O\email_detials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5552E9E5-38CB-4B3C-9E95-CEA941D8ACBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC0DB0A-2354-4600-8932-91D6198893CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>NucleusTeq</t>
   </si>
@@ -43,39 +43,24 @@
     <t>Full Name</t>
   </si>
   <si>
-    <t>N0165</t>
-  </si>
-  <si>
     <t>Mandal</t>
   </si>
   <si>
     <t>Diksha Mandal</t>
   </si>
   <si>
-    <t>N0163</t>
-  </si>
-  <si>
-    <t>Sajal</t>
-  </si>
-  <si>
     <t>Nema</t>
   </si>
   <si>
     <t>Sajal Nema</t>
   </si>
   <si>
-    <t>N0094</t>
-  </si>
-  <si>
     <t>Kale</t>
   </si>
   <si>
     <t>Shantanu Kale</t>
   </si>
   <si>
-    <t>nemasajal13@gmail.com</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
@@ -95,6 +80,18 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>N0262</t>
+  </si>
+  <si>
+    <t>Satbeer Singh Bhatia</t>
+  </si>
+  <si>
+    <t>anil.vishwakarma998135@gmail.com</t>
+  </si>
+  <si>
+    <t>N0285</t>
   </si>
 </sst>
 </file>
@@ -536,7 +533,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>3</v>
@@ -551,75 +548,69 @@
         <v>6</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="F5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>17</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="3"/>
+        <v>21</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="G8" s="3"/>
@@ -636,7 +627,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C14" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -648,7 +639,7 @@
   <hyperlinks>
     <hyperlink ref="G6" r:id="rId1" xr:uid="{8F63C5F2-14D9-412F-8876-C79027429007}"/>
     <hyperlink ref="G4" r:id="rId2" xr:uid="{57B98DEC-E897-4907-AECA-6DEE762020A3}"/>
-    <hyperlink ref="G5" r:id="rId3" xr:uid="{FB981B75-912E-475A-AE17-B074F175BEA4}"/>
+    <hyperlink ref="G7" r:id="rId3" xr:uid="{0998B3F2-E2A8-47AF-AFBE-C100D192C110}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>

</xml_diff>